<commit_message>
Fix Cubs 2026-03-28: game location (Wrigley not Nationals Park) and game number (2 not 3)
Opening Day was at Wrigley Field, not Washington. Today is Game 2, not Game 3.
Corrected across all content files and regenerated PostPlanner export.

https://claude.ai/code/session_01GLzGWEPr2e7Y4v9NhULCZ6
</commit_message>
<xml_diff>
--- a/Cubs/postplanner-imports/cubs-postplanner-2026-03-28.xlsx
+++ b/Cubs/postplanner-imports/cubs-postplanner-2026-03-28.xlsx
@@ -478,7 +478,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>03/28/2026  11:22</t>
+          <t>03/28/2026  11:40</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -493,7 +493,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>03/28/2026  12:32</t>
+          <t>03/28/2026  12:48</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -508,7 +508,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>03/28/2026  13:42</t>
+          <t>03/28/2026  13:56</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -523,7 +523,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03/28/2026  14:52</t>
+          <t>03/28/2026  15:04</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -538,7 +538,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>03/28/2026  16:02</t>
+          <t>03/28/2026  16:12</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -553,7 +553,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>03/28/2026  17:12</t>
+          <t>03/28/2026  17:20</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -570,12 +570,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>03/28/2026  18:22</t>
+          <t>03/28/2026  18:28</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Cade Horton takes the mound tonight for Game 3.
+          <t>Cade Horton takes the mound tonight for Game 2.
 He went 11-4 with a 2.67 ERA as a ROOKIE in 2025. This is the guy the Cubs built around.
 Miles Mikolas better be ready. 🔥
 #Cubs #GoCubs #FlyTheW</t>
@@ -585,13 +585,13 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>03/28/2026  19:32</t>
+          <t>03/28/2026  19:36</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
           <t>First pitch in minutes.
-Cade Horton. Nationals Park. Win or go home on this road trip.
+Cade Horton. Wrigley Field. Chance to even the series at home.
 Let's go, Cubs.
 #Cubs #GoCubs #FlyTheW</t>
         </is>
@@ -600,7 +600,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>03/28/2026  20:42</t>
+          <t>03/28/2026  20:44</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">

</xml_diff>